<commit_message>
fix: remove mergeCells from excel signature block to prevent template collision
</commit_message>
<xml_diff>
--- a/public/templates/template_arsip_masuk.xlsx
+++ b/public/templates/template_arsip_masuk.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\.gemini\antigravity\scratch\bidi-dlh-app\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F680C7F5-6E76-45C6-8C5E-8E5F518ED121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6817FC8C-20B7-4254-B886-E50867FAD1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{D506533D-B42B-4478-B220-342326BBDD67}"/>
+    <workbookView xWindow="2415" yWindow="2685" windowWidth="21600" windowHeight="11295" xr2:uid="{D506533D-B42B-4478-B220-342326BBDD67}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -91,7 +91,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="175" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="164" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -343,7 +343,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="175" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -358,7 +358,7 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="175" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -367,7 +367,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="175" fontId="2" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -382,13 +382,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="175" fontId="2" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="175" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="175" fontId="2" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -397,22 +397,22 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="175" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="175" fontId="3" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="175" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -442,18 +442,27 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -478,23 +487,14 @@
     <xf numFmtId="49" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="175" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -827,52 +827,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-      <c r="H1" s="56"/>
-      <c r="I1" s="56"/>
-      <c r="J1" s="56"/>
-      <c r="K1" s="56"/>
-      <c r="L1" s="56"/>
-      <c r="M1" s="56"/>
-      <c r="N1" s="56"/>
-      <c r="O1" s="56"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
+      <c r="J1" s="44"/>
+      <c r="K1" s="44"/>
+      <c r="L1" s="44"/>
+      <c r="M1" s="44"/>
+      <c r="N1" s="44"/>
+      <c r="O1" s="44"/>
     </row>
     <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="57"/>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
-      <c r="F2" s="57"/>
-      <c r="G2" s="57"/>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
-      <c r="L2" s="57"/>
-      <c r="M2" s="57"/>
-      <c r="N2" s="57"/>
-      <c r="O2" s="57"/>
+      <c r="A2" s="45"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
     </row>
     <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="58" t="s">
+      <c r="A4" s="46" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="58"/>
-      <c r="C4" s="58"/>
-      <c r="D4" s="58"/>
-      <c r="E4" s="58"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="58"/>
-      <c r="H4" s="58"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
       <c r="I4" s="11"/>
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
@@ -916,49 +916,49 @@
       <c r="O6" s="5"/>
     </row>
     <row r="7" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="59" t="s">
+      <c r="A7" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="59" t="s">
+      <c r="C7" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="50" t="s">
+      <c r="D7" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
-      <c r="G7" s="52"/>
-      <c r="H7" s="59" t="s">
+      <c r="E7" s="54"/>
+      <c r="F7" s="54"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="47" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="60" t="s">
+      <c r="I7" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="J7" s="61" t="s">
+      <c r="J7" s="49" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="59" t="s">
+      <c r="K7" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="L7" s="59"/>
-      <c r="M7" s="59"/>
-      <c r="N7" s="59"/>
-      <c r="O7" s="59"/>
+      <c r="L7" s="47"/>
+      <c r="M7" s="47"/>
+      <c r="N7" s="47"/>
+      <c r="O7" s="47"/>
     </row>
     <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="59"/>
-      <c r="B8" s="49"/>
-      <c r="C8" s="59"/>
-      <c r="D8" s="53"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="55"/>
-      <c r="H8" s="59"/>
-      <c r="I8" s="60"/>
-      <c r="J8" s="61"/>
+      <c r="A8" s="47"/>
+      <c r="B8" s="52"/>
+      <c r="C8" s="47"/>
+      <c r="D8" s="56"/>
+      <c r="E8" s="57"/>
+      <c r="F8" s="57"/>
+      <c r="G8" s="58"/>
+      <c r="H8" s="47"/>
+      <c r="I8" s="48"/>
+      <c r="J8" s="49"/>
       <c r="K8" s="15" t="s">
         <v>8</v>
       </c>
@@ -1019,12 +1019,12 @@
       <c r="G11" s="21"/>
       <c r="H11" s="18"/>
       <c r="I11" s="19"/>
-      <c r="J11" s="46"/>
-      <c r="K11" s="46"/>
-      <c r="L11" s="46"/>
-      <c r="M11" s="46"/>
-      <c r="N11" s="46"/>
-      <c r="O11" s="46"/>
+      <c r="J11" s="60"/>
+      <c r="K11" s="60"/>
+      <c r="L11" s="60"/>
+      <c r="M11" s="60"/>
+      <c r="N11" s="60"/>
+      <c r="O11" s="60"/>
     </row>
     <row r="12" spans="1:15" s="43" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
@@ -1036,12 +1036,12 @@
       <c r="G12" s="21"/>
       <c r="H12" s="18"/>
       <c r="I12" s="19"/>
-      <c r="J12" s="47"/>
-      <c r="K12" s="47"/>
-      <c r="L12" s="47"/>
-      <c r="M12" s="47"/>
-      <c r="N12" s="47"/>
-      <c r="O12" s="47"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="59"/>
+      <c r="L12" s="59"/>
+      <c r="M12" s="59"/>
+      <c r="N12" s="59"/>
+      <c r="O12" s="59"/>
     </row>
     <row r="13" spans="1:15" s="43" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
@@ -1104,12 +1104,12 @@
       <c r="G16" s="21"/>
       <c r="H16" s="18"/>
       <c r="I16" s="19"/>
-      <c r="J16" s="44"/>
-      <c r="K16" s="44"/>
-      <c r="L16" s="44"/>
-      <c r="M16" s="44"/>
-      <c r="N16" s="44"/>
-      <c r="O16" s="44"/>
+      <c r="J16" s="61"/>
+      <c r="K16" s="61"/>
+      <c r="L16" s="61"/>
+      <c r="M16" s="61"/>
+      <c r="N16" s="61"/>
+      <c r="O16" s="61"/>
     </row>
     <row r="17" spans="1:15" s="43" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
@@ -1121,12 +1121,12 @@
       <c r="G17" s="21"/>
       <c r="H17" s="18"/>
       <c r="I17" s="19"/>
-      <c r="J17" s="45"/>
-      <c r="K17" s="45"/>
-      <c r="L17" s="45"/>
-      <c r="M17" s="45"/>
-      <c r="N17" s="45"/>
-      <c r="O17" s="45"/>
+      <c r="J17" s="50"/>
+      <c r="K17" s="50"/>
+      <c r="L17" s="50"/>
+      <c r="M17" s="50"/>
+      <c r="N17" s="50"/>
+      <c r="O17" s="50"/>
     </row>
     <row r="18" spans="1:15" s="43" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
@@ -5641,7 +5641,10 @@
       <c r="AO342" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="12">
+    <mergeCell ref="J17:O17"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="D7:G8"/>
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A2:O2"/>
     <mergeCell ref="A4:H4"/>
@@ -5651,12 +5654,6 @@
     <mergeCell ref="I7:I8"/>
     <mergeCell ref="J7:J8"/>
     <mergeCell ref="K7:O7"/>
-    <mergeCell ref="J16:O16"/>
-    <mergeCell ref="J17:O17"/>
-    <mergeCell ref="J11:O11"/>
-    <mergeCell ref="J12:O12"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="D7:G8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="46" fitToHeight="0" orientation="landscape" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>

</xml_diff>

<commit_message>
fix: force signature block merges to ensure consistent width between name and nip
</commit_message>
<xml_diff>
--- a/public/templates/template_arsip_masuk.xlsx
+++ b/public/templates/template_arsip_masuk.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\.gemini\antigravity\scratch\bidi-dlh-app\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6817FC8C-20B7-4254-B886-E50867FAD1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6B20C06-12B2-4FAC-A845-E259712F76BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2415" yWindow="2685" windowWidth="21600" windowHeight="11295" xr2:uid="{D506533D-B42B-4478-B220-342326BBDD67}"/>
+    <workbookView xWindow="2070" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{D506533D-B42B-4478-B220-342326BBDD67}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -442,6 +442,39 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -461,39 +494,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -827,52 +827,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="55" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
-      <c r="J1" s="44"/>
-      <c r="K1" s="44"/>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
+      <c r="B1" s="55"/>
+      <c r="C1" s="55"/>
+      <c r="D1" s="55"/>
+      <c r="E1" s="55"/>
+      <c r="F1" s="55"/>
+      <c r="G1" s="55"/>
+      <c r="H1" s="55"/>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="55"/>
+      <c r="L1" s="55"/>
+      <c r="M1" s="55"/>
+      <c r="N1" s="55"/>
+      <c r="O1" s="55"/>
     </row>
     <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="45"/>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
-      <c r="K2" s="45"/>
-      <c r="L2" s="45"/>
-      <c r="M2" s="45"/>
-      <c r="N2" s="45"/>
-      <c r="O2" s="45"/>
+      <c r="A2" s="56"/>
+      <c r="B2" s="56"/>
+      <c r="C2" s="56"/>
+      <c r="D2" s="56"/>
+      <c r="E2" s="56"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
+      <c r="J2" s="56"/>
+      <c r="K2" s="56"/>
+      <c r="L2" s="56"/>
+      <c r="M2" s="56"/>
+      <c r="N2" s="56"/>
+      <c r="O2" s="56"/>
     </row>
     <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
-      <c r="H4" s="46"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
       <c r="I4" s="11"/>
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
@@ -916,49 +916,49 @@
       <c r="O6" s="5"/>
     </row>
     <row r="7" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="47" t="s">
+      <c r="A7" s="58" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="51" t="s">
+      <c r="B7" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="47" t="s">
+      <c r="C7" s="58" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="53" t="s">
+      <c r="D7" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="55"/>
-      <c r="H7" s="47" t="s">
+      <c r="E7" s="50"/>
+      <c r="F7" s="50"/>
+      <c r="G7" s="51"/>
+      <c r="H7" s="58" t="s">
         <v>4</v>
       </c>
-      <c r="I7" s="48" t="s">
+      <c r="I7" s="59" t="s">
         <v>5</v>
       </c>
-      <c r="J7" s="49" t="s">
+      <c r="J7" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="K7" s="47" t="s">
+      <c r="K7" s="58" t="s">
         <v>7</v>
       </c>
-      <c r="L7" s="47"/>
-      <c r="M7" s="47"/>
-      <c r="N7" s="47"/>
-      <c r="O7" s="47"/>
+      <c r="L7" s="58"/>
+      <c r="M7" s="58"/>
+      <c r="N7" s="58"/>
+      <c r="O7" s="58"/>
     </row>
     <row r="8" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="47"/>
-      <c r="B8" s="52"/>
-      <c r="C8" s="47"/>
-      <c r="D8" s="56"/>
-      <c r="E8" s="57"/>
-      <c r="F8" s="57"/>
-      <c r="G8" s="58"/>
-      <c r="H8" s="47"/>
-      <c r="I8" s="48"/>
-      <c r="J8" s="49"/>
+      <c r="A8" s="58"/>
+      <c r="B8" s="48"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="52"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="53"/>
+      <c r="G8" s="54"/>
+      <c r="H8" s="58"/>
+      <c r="I8" s="59"/>
+      <c r="J8" s="60"/>
       <c r="K8" s="15" t="s">
         <v>8</v>
       </c>
@@ -1019,12 +1019,12 @@
       <c r="G11" s="21"/>
       <c r="H11" s="18"/>
       <c r="I11" s="19"/>
-      <c r="J11" s="60"/>
-      <c r="K11" s="60"/>
-      <c r="L11" s="60"/>
-      <c r="M11" s="60"/>
-      <c r="N11" s="60"/>
-      <c r="O11" s="60"/>
+      <c r="J11" s="45"/>
+      <c r="K11" s="45"/>
+      <c r="L11" s="45"/>
+      <c r="M11" s="45"/>
+      <c r="N11" s="45"/>
+      <c r="O11" s="45"/>
     </row>
     <row r="12" spans="1:15" s="43" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8"/>
@@ -1036,12 +1036,12 @@
       <c r="G12" s="21"/>
       <c r="H12" s="18"/>
       <c r="I12" s="19"/>
-      <c r="J12" s="59"/>
-      <c r="K12" s="59"/>
-      <c r="L12" s="59"/>
-      <c r="M12" s="59"/>
-      <c r="N12" s="59"/>
-      <c r="O12" s="59"/>
+      <c r="J12" s="44"/>
+      <c r="K12" s="44"/>
+      <c r="L12" s="44"/>
+      <c r="M12" s="44"/>
+      <c r="N12" s="44"/>
+      <c r="O12" s="44"/>
     </row>
     <row r="13" spans="1:15" s="43" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="8"/>
@@ -1070,8 +1070,6 @@
       <c r="G14" s="21"/>
       <c r="H14" s="18"/>
       <c r="I14" s="19"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
       <c r="L14" s="23"/>
       <c r="M14" s="23"/>
       <c r="N14" s="23"/>
@@ -1104,12 +1102,12 @@
       <c r="G16" s="21"/>
       <c r="H16" s="18"/>
       <c r="I16" s="19"/>
-      <c r="J16" s="61"/>
-      <c r="K16" s="61"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="61"/>
-      <c r="N16" s="61"/>
-      <c r="O16" s="61"/>
+      <c r="J16" s="46"/>
+      <c r="K16" s="46"/>
+      <c r="L16" s="46"/>
+      <c r="M16" s="46"/>
+      <c r="N16" s="46"/>
+      <c r="O16" s="46"/>
     </row>
     <row r="17" spans="1:15" s="43" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="8"/>
@@ -1121,12 +1119,12 @@
       <c r="G17" s="21"/>
       <c r="H17" s="18"/>
       <c r="I17" s="19"/>
-      <c r="J17" s="50"/>
-      <c r="K17" s="50"/>
-      <c r="L17" s="50"/>
-      <c r="M17" s="50"/>
-      <c r="N17" s="50"/>
-      <c r="O17" s="50"/>
+      <c r="J17" s="61"/>
+      <c r="K17" s="61"/>
+      <c r="L17" s="61"/>
+      <c r="M17" s="61"/>
+      <c r="N17" s="61"/>
+      <c r="O17" s="61"/>
     </row>
     <row r="18" spans="1:15" s="43" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="8"/>
@@ -5641,8 +5639,7 @@
       <c r="AO342" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="J17:O17"/>
+  <mergeCells count="11">
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="D7:G8"/>
     <mergeCell ref="A1:O1"/>

</xml_diff>